<commit_message>
Update Ferahlatıcılar prices; Premium Soda → San Pellegrino
</commit_message>
<xml_diff>
--- a/menu/Ciao_Fiyat_Listesi.xlsx
+++ b/menu/Ciao_Fiyat_Listesi.xlsx
@@ -668,7 +668,7 @@
     <t xml:space="preserve">Soda</t>
   </si>
   <si>
-    <t xml:space="preserve">Premium Soda</t>
+    <t xml:space="preserve">San Pellegrino</t>
   </si>
   <si>
     <t xml:space="preserve">Limonata</t>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="C59" s="24"/>
       <c r="D59" s="25" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="E59" s="25"/>
       <c r="F59" s="36"/>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C60" s="24"/>
       <c r="D60" s="25" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E60" s="25"/>
       <c r="F60" s="36"/>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="C61" s="24"/>
       <c r="D61" s="25" t="n">
-        <v>100</v>
+        <v>170</v>
       </c>
       <c r="E61" s="25"/>
       <c r="F61" s="36"/>
@@ -3857,7 +3857,7 @@
       </c>
       <c r="C62" s="24"/>
       <c r="D62" s="25" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="E62" s="25"/>
       <c r="F62" s="36"/>
@@ -7154,7 +7154,7 @@
       <c r="F85" s="45"/>
       <c r="G85" s="47" t="n">
         <f aca="false">IF(Soğuklar!D59="","",Soğuklar!D59)</f>
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="H85" s="47"/>
       <c r="I85" s="47"/>
@@ -7163,7 +7163,7 @@
       <c r="L85" s="45"/>
       <c r="M85" s="48" t="n">
         <f aca="false">IF(COUNT(G85:I85)=0,"",MIN(G85:I85))</f>
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7180,7 +7180,7 @@
       <c r="F86" s="45"/>
       <c r="G86" s="47" t="n">
         <f aca="false">IF(Soğuklar!D60="","",Soğuklar!D60)</f>
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="H86" s="47"/>
       <c r="I86" s="47"/>
@@ -7189,7 +7189,7 @@
       <c r="L86" s="45"/>
       <c r="M86" s="48" t="n">
         <f aca="false">IF(COUNT(G86:I86)=0,"",MIN(G86:I86))</f>
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7206,7 +7206,7 @@
       <c r="F87" s="45"/>
       <c r="G87" s="47" t="n">
         <f aca="false">IF(Soğuklar!D61="","",Soğuklar!D61)</f>
-        <v>100</v>
+        <v>170</v>
       </c>
       <c r="H87" s="47"/>
       <c r="I87" s="47"/>
@@ -7215,7 +7215,7 @@
       <c r="L87" s="45"/>
       <c r="M87" s="48" t="n">
         <f aca="false">IF(COUNT(G87:I87)=0,"",MIN(G87:I87))</f>
-        <v>100</v>
+        <v>170</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7232,7 +7232,7 @@
       <c r="F88" s="45"/>
       <c r="G88" s="47" t="n">
         <f aca="false">IF(Soğuklar!D62="","",Soğuklar!D62)</f>
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="H88" s="47"/>
       <c r="I88" s="47"/>
@@ -7241,7 +7241,7 @@
       <c r="L88" s="45"/>
       <c r="M88" s="48" t="n">
         <f aca="false">IF(COUNT(G88:I88)=0,"",MIN(G88:I88))</f>
-        <v>130</v>
+        <v>200</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
7x4 cm price labels and 7x12 cm tea labels
</commit_message>
<xml_diff>
--- a/menu/Ciao_Fiyat_Listesi.xlsx
+++ b/menu/Ciao_Fiyat_Listesi.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1914" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1920" uniqueCount="350">
   <si>
     <t xml:space="preserve">MENÜ FİYAT LİSTESİ</t>
   </si>
@@ -915,7 +915,7 @@
     <t xml:space="preserve">Fiyat Soğuklar sayfasından gelir</t>
   </si>
   <si>
-    <t xml:space="preserve">Bu ürünlerin hepsinin 8 × 5 cm fiyat etiketi vardır. Mavi rakamlar burada girilir; yeşil rakamlar Soğuklar sayfasından gelir.</t>
+    <t xml:space="preserve">Bu ürünlerin hepsinin 7 × 4 cm fiyat etiketi vardır. Mavi rakamlar burada girilir; yeşil rakamlar Soğuklar sayfasından gelir.</t>
   </si>
   <si>
     <t xml:space="preserve">TÜM ÜRÜNLER · POS</t>
@@ -1011,6 +1011,9 @@
     <t xml:space="preserve">Kasa (ekranda yok)</t>
   </si>
   <si>
+    <t xml:space="preserve">Var</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ciao Signature</t>
   </si>
   <si>
@@ -1045,9 +1048,6 @@
   </si>
   <si>
     <t xml:space="preserve">Ekran 2 · Bar önü</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Var</t>
   </si>
   <si>
     <t xml:space="preserve">Tatlılar</t>
@@ -10035,7 +10035,9 @@
       <c r="H59" s="58" t="s">
         <v>319</v>
       </c>
-      <c r="I59" s="60"/>
+      <c r="I59" s="60" t="s">
+        <v>325</v>
+      </c>
       <c r="J59" s="58"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10061,7 +10063,9 @@
       <c r="H60" s="58" t="s">
         <v>319</v>
       </c>
-      <c r="I60" s="60"/>
+      <c r="I60" s="60" t="s">
+        <v>325</v>
+      </c>
       <c r="J60" s="58"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10087,7 +10091,9 @@
       <c r="H61" s="58" t="s">
         <v>319</v>
       </c>
-      <c r="I61" s="60"/>
+      <c r="I61" s="60" t="s">
+        <v>325</v>
+      </c>
       <c r="J61" s="58"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10113,7 +10119,9 @@
       <c r="H62" s="58" t="s">
         <v>319</v>
       </c>
-      <c r="I62" s="60"/>
+      <c r="I62" s="60" t="s">
+        <v>325</v>
+      </c>
       <c r="J62" s="58"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10139,7 +10147,9 @@
       <c r="H63" s="58" t="s">
         <v>319</v>
       </c>
-      <c r="I63" s="60"/>
+      <c r="I63" s="60" t="s">
+        <v>325</v>
+      </c>
       <c r="J63" s="58"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10165,7 +10175,9 @@
       <c r="H64" s="58" t="s">
         <v>319</v>
       </c>
-      <c r="I64" s="60"/>
+      <c r="I64" s="60" t="s">
+        <v>325</v>
+      </c>
       <c r="J64" s="58"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10173,7 +10185,7 @@
         <v>317</v>
       </c>
       <c r="C65" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D65" s="59" t="s">
         <v>116</v>
@@ -10199,7 +10211,7 @@
         <v>317</v>
       </c>
       <c r="C66" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D66" s="59" t="s">
         <v>116</v>
@@ -10225,7 +10237,7 @@
         <v>317</v>
       </c>
       <c r="C67" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D67" s="59" t="s">
         <v>119</v>
@@ -10251,7 +10263,7 @@
         <v>317</v>
       </c>
       <c r="C68" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D68" s="59" t="s">
         <v>119</v>
@@ -10277,7 +10289,7 @@
         <v>317</v>
       </c>
       <c r="C69" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D69" s="59" t="s">
         <v>121</v>
@@ -10303,7 +10315,7 @@
         <v>317</v>
       </c>
       <c r="C70" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D70" s="59" t="s">
         <v>121</v>
@@ -10329,7 +10341,7 @@
         <v>317</v>
       </c>
       <c r="C71" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D71" s="59" t="s">
         <v>123</v>
@@ -10355,7 +10367,7 @@
         <v>317</v>
       </c>
       <c r="C72" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D72" s="59" t="s">
         <v>123</v>
@@ -10381,7 +10393,7 @@
         <v>317</v>
       </c>
       <c r="C73" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D73" s="59" t="s">
         <v>125</v>
@@ -10407,7 +10419,7 @@
         <v>317</v>
       </c>
       <c r="C74" s="58" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D74" s="59" t="s">
         <v>125</v>
@@ -10430,10 +10442,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="57" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C75" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D75" s="59" t="s">
         <v>137</v>
@@ -10449,17 +10461,17 @@
         <v>170</v>
       </c>
       <c r="H75" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I75" s="60"/>
       <c r="J75" s="58"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C76" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D76" s="59" t="s">
         <v>137</v>
@@ -10475,17 +10487,17 @@
         <v>190</v>
       </c>
       <c r="H76" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I76" s="60"/>
       <c r="J76" s="58"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C77" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D77" s="59" t="s">
         <v>139</v>
@@ -10501,17 +10513,17 @@
         <v>220</v>
       </c>
       <c r="H77" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I77" s="60"/>
       <c r="J77" s="58"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C78" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D78" s="59" t="s">
         <v>139</v>
@@ -10527,17 +10539,17 @@
         <v>240</v>
       </c>
       <c r="H78" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I78" s="60"/>
       <c r="J78" s="58"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C79" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D79" s="59" t="s">
         <v>141</v>
@@ -10553,17 +10565,17 @@
         <v>240</v>
       </c>
       <c r="H79" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I79" s="60"/>
       <c r="J79" s="58"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C80" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D80" s="59" t="s">
         <v>141</v>
@@ -10579,17 +10591,17 @@
         <v>260</v>
       </c>
       <c r="H80" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I80" s="60"/>
       <c r="J80" s="58"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C81" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D81" s="59" t="s">
         <v>143</v>
@@ -10605,17 +10617,17 @@
         <v>230</v>
       </c>
       <c r="H81" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I81" s="60"/>
       <c r="J81" s="58"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C82" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D82" s="59" t="s">
         <v>143</v>
@@ -10631,17 +10643,17 @@
         <v>250</v>
       </c>
       <c r="H82" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I82" s="60"/>
       <c r="J82" s="58"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C83" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D83" s="59" t="s">
         <v>145</v>
@@ -10657,17 +10669,17 @@
         <v>250</v>
       </c>
       <c r="H83" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I83" s="60"/>
       <c r="J83" s="58"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C84" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D84" s="59" t="s">
         <v>145</v>
@@ -10683,17 +10695,17 @@
         <v>280</v>
       </c>
       <c r="H84" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I84" s="60"/>
       <c r="J84" s="58"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C85" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D85" s="59" t="s">
         <v>147</v>
@@ -10709,17 +10721,17 @@
         <v>150</v>
       </c>
       <c r="H85" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I85" s="60"/>
       <c r="J85" s="58"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C86" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D86" s="59" t="s">
         <v>147</v>
@@ -10735,17 +10747,17 @@
         <v>170</v>
       </c>
       <c r="H86" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I86" s="60"/>
       <c r="J86" s="58"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C87" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D87" s="59" t="s">
         <v>149</v>
@@ -10761,17 +10773,17 @@
         <v>250</v>
       </c>
       <c r="H87" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I87" s="60"/>
       <c r="J87" s="58"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C88" s="58" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D88" s="59" t="s">
         <v>149</v>
@@ -10787,17 +10799,17 @@
         <v>270</v>
       </c>
       <c r="H88" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I88" s="60"/>
       <c r="J88" s="58"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C89" s="58" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D89" s="59" t="s">
         <v>152</v>
@@ -10813,17 +10825,17 @@
         <v>150</v>
       </c>
       <c r="H89" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I89" s="60"/>
       <c r="J89" s="58"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C90" s="58" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D90" s="59" t="s">
         <v>152</v>
@@ -10839,17 +10851,17 @@
         <v>170</v>
       </c>
       <c r="H90" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I90" s="60"/>
       <c r="J90" s="58"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C91" s="58" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D91" s="59" t="s">
         <v>154</v>
@@ -10865,17 +10877,17 @@
         <v>170</v>
       </c>
       <c r="H91" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I91" s="60"/>
       <c r="J91" s="58"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C92" s="58" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D92" s="59" t="s">
         <v>154</v>
@@ -10891,14 +10903,14 @@
         <v>190</v>
       </c>
       <c r="H92" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I92" s="60"/>
       <c r="J92" s="58"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C93" s="58" t="s">
         <v>157</v>
@@ -10917,14 +10929,14 @@
         <v>170</v>
       </c>
       <c r="H93" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I93" s="60"/>
       <c r="J93" s="58"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C94" s="58" t="s">
         <v>157</v>
@@ -10943,17 +10955,17 @@
         <v>190</v>
       </c>
       <c r="H94" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I94" s="60"/>
       <c r="J94" s="58"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C95" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D95" s="59" t="s">
         <v>160</v>
@@ -10969,17 +10981,17 @@
         <v>250</v>
       </c>
       <c r="H95" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I95" s="60"/>
       <c r="J95" s="58"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C96" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D96" s="59" t="s">
         <v>160</v>
@@ -10995,17 +11007,17 @@
         <v>270</v>
       </c>
       <c r="H96" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I96" s="60"/>
       <c r="J96" s="58"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C97" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D97" s="59" t="s">
         <v>161</v>
@@ -11021,17 +11033,17 @@
         <v>250</v>
       </c>
       <c r="H97" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I97" s="60"/>
       <c r="J97" s="58"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C98" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D98" s="59" t="s">
         <v>161</v>
@@ -11047,17 +11059,17 @@
         <v>270</v>
       </c>
       <c r="H98" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I98" s="60"/>
       <c r="J98" s="58"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C99" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D99" s="59" t="s">
         <v>163</v>
@@ -11073,17 +11085,17 @@
         <v>250</v>
       </c>
       <c r="H99" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I99" s="60"/>
       <c r="J99" s="58"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C100" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D100" s="59" t="s">
         <v>163</v>
@@ -11099,17 +11111,17 @@
         <v>270</v>
       </c>
       <c r="H100" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I100" s="60"/>
       <c r="J100" s="58"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C101" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D101" s="59" t="s">
         <v>165</v>
@@ -11125,17 +11137,17 @@
         <v>240</v>
       </c>
       <c r="H101" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I101" s="60"/>
       <c r="J101" s="58"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C102" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D102" s="59" t="s">
         <v>165</v>
@@ -11151,17 +11163,17 @@
         <v>260</v>
       </c>
       <c r="H102" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I102" s="60"/>
       <c r="J102" s="58"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B103" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C103" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D103" s="59" t="s">
         <v>167</v>
@@ -11177,17 +11189,17 @@
         <v>260</v>
       </c>
       <c r="H103" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I103" s="60"/>
       <c r="J103" s="58"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C104" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D104" s="59" t="s">
         <v>167</v>
@@ -11203,17 +11215,17 @@
         <v>280</v>
       </c>
       <c r="H104" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I104" s="60"/>
       <c r="J104" s="58"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C105" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D105" s="59" t="s">
         <v>169</v>
@@ -11229,17 +11241,17 @@
         <v>300</v>
       </c>
       <c r="H105" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I105" s="60"/>
       <c r="J105" s="58"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B106" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C106" s="58" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D106" s="59" t="s">
         <v>169</v>
@@ -11255,17 +11267,17 @@
         <v>340</v>
       </c>
       <c r="H106" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I106" s="60"/>
       <c r="J106" s="58"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C107" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D107" s="59" t="s">
         <v>172</v>
@@ -11281,17 +11293,17 @@
         <v>280</v>
       </c>
       <c r="H107" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I107" s="60"/>
       <c r="J107" s="58"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C108" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D108" s="59" t="s">
         <v>172</v>
@@ -11307,17 +11319,17 @@
         <v>300</v>
       </c>
       <c r="H108" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I108" s="60"/>
       <c r="J108" s="58"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C109" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D109" s="59" t="s">
         <v>174</v>
@@ -11333,17 +11345,17 @@
         <v>270</v>
       </c>
       <c r="H109" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I109" s="60"/>
       <c r="J109" s="58"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C110" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D110" s="59" t="s">
         <v>174</v>
@@ -11359,17 +11371,17 @@
         <v>290</v>
       </c>
       <c r="H110" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I110" s="60"/>
       <c r="J110" s="58"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B111" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C111" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D111" s="59" t="s">
         <v>176</v>
@@ -11385,17 +11397,17 @@
         <v>270</v>
       </c>
       <c r="H111" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I111" s="60"/>
       <c r="J111" s="58"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C112" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D112" s="59" t="s">
         <v>176</v>
@@ -11411,17 +11423,17 @@
         <v>290</v>
       </c>
       <c r="H112" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I112" s="60"/>
       <c r="J112" s="58"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C113" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D113" s="59" t="s">
         <v>178</v>
@@ -11437,17 +11449,17 @@
         <v>300</v>
       </c>
       <c r="H113" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I113" s="60"/>
       <c r="J113" s="58"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C114" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D114" s="59" t="s">
         <v>178</v>
@@ -11463,17 +11475,17 @@
         <v>320</v>
       </c>
       <c r="H114" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I114" s="60"/>
       <c r="J114" s="58"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C115" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D115" s="59" t="s">
         <v>180</v>
@@ -11489,17 +11501,17 @@
         <v>300</v>
       </c>
       <c r="H115" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I115" s="60"/>
       <c r="J115" s="58"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C116" s="58" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D116" s="59" t="s">
         <v>180</v>
@@ -11515,17 +11527,17 @@
         <v>320</v>
       </c>
       <c r="H116" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I116" s="60"/>
       <c r="J116" s="58"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C117" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D117" s="59" t="s">
         <v>183</v>
@@ -11541,17 +11553,17 @@
         <v>260</v>
       </c>
       <c r="H117" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I117" s="60"/>
       <c r="J117" s="58"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B118" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C118" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D118" s="59" t="s">
         <v>183</v>
@@ -11567,17 +11579,17 @@
         <v>280</v>
       </c>
       <c r="H118" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I118" s="60"/>
       <c r="J118" s="58"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B119" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C119" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D119" s="59" t="s">
         <v>185</v>
@@ -11593,17 +11605,17 @@
         <v>260</v>
       </c>
       <c r="H119" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I119" s="60"/>
       <c r="J119" s="58"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C120" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D120" s="59" t="s">
         <v>185</v>
@@ -11619,17 +11631,17 @@
         <v>280</v>
       </c>
       <c r="H120" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I120" s="60"/>
       <c r="J120" s="58"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C121" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D121" s="59" t="s">
         <v>186</v>
@@ -11645,17 +11657,17 @@
         <v>240</v>
       </c>
       <c r="H121" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I121" s="60"/>
       <c r="J121" s="58"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C122" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D122" s="59" t="s">
         <v>186</v>
@@ -11671,17 +11683,17 @@
         <v>260</v>
       </c>
       <c r="H122" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I122" s="60"/>
       <c r="J122" s="58"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C123" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D123" s="59" t="s">
         <v>188</v>
@@ -11697,17 +11709,17 @@
         <v>270</v>
       </c>
       <c r="H123" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I123" s="60"/>
       <c r="J123" s="58"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C124" s="58" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D124" s="59" t="s">
         <v>188</v>
@@ -11723,17 +11735,17 @@
         <v>290</v>
       </c>
       <c r="H124" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I124" s="60"/>
       <c r="J124" s="58"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C125" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D125" s="59" t="s">
         <v>191</v>
@@ -11749,17 +11761,17 @@
         <v>300</v>
       </c>
       <c r="H125" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I125" s="60"/>
       <c r="J125" s="58"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C126" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D126" s="59" t="s">
         <v>191</v>
@@ -11775,17 +11787,17 @@
         <v>320</v>
       </c>
       <c r="H126" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I126" s="60"/>
       <c r="J126" s="58"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C127" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D127" s="59" t="s">
         <v>193</v>
@@ -11801,17 +11813,17 @@
         <v>330</v>
       </c>
       <c r="H127" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I127" s="60"/>
       <c r="J127" s="58"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B128" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C128" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D128" s="59" t="s">
         <v>193</v>
@@ -11827,17 +11839,17 @@
         <v>350</v>
       </c>
       <c r="H128" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I128" s="60"/>
       <c r="J128" s="58"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B129" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C129" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D129" s="59" t="s">
         <v>195</v>
@@ -11853,17 +11865,17 @@
         <v>290</v>
       </c>
       <c r="H129" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I129" s="60"/>
       <c r="J129" s="58"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C130" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D130" s="59" t="s">
         <v>195</v>
@@ -11879,17 +11891,17 @@
         <v>310</v>
       </c>
       <c r="H130" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I130" s="60"/>
       <c r="J130" s="58"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C131" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D131" s="59" t="s">
         <v>197</v>
@@ -11905,17 +11917,17 @@
         <v>290</v>
       </c>
       <c r="H131" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I131" s="60"/>
       <c r="J131" s="58"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C132" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D132" s="59" t="s">
         <v>197</v>
@@ -11931,17 +11943,17 @@
         <v>310</v>
       </c>
       <c r="H132" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I132" s="60"/>
       <c r="J132" s="58"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C133" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D133" s="59" t="s">
         <v>199</v>
@@ -11957,17 +11969,17 @@
         <v>290</v>
       </c>
       <c r="H133" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I133" s="60"/>
       <c r="J133" s="58"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="61" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C134" s="58" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D134" s="59" t="s">
         <v>199</v>
@@ -11983,17 +11995,17 @@
         <v>310</v>
       </c>
       <c r="H134" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I134" s="60"/>
       <c r="J134" s="58"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C135" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C135" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D135" s="59" t="s">
         <v>116</v>
@@ -12009,17 +12021,17 @@
         <v>300</v>
       </c>
       <c r="H135" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I135" s="60"/>
       <c r="J135" s="58"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B136" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C136" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C136" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D136" s="59" t="s">
         <v>116</v>
@@ -12035,17 +12047,17 @@
         <v>320</v>
       </c>
       <c r="H136" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I136" s="60"/>
       <c r="J136" s="58"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B137" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C137" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C137" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D137" s="59" t="s">
         <v>202</v>
@@ -12061,7 +12073,7 @@
         <v>280</v>
       </c>
       <c r="H137" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I137" s="60"/>
       <c r="J137" s="58" t="s">
@@ -12070,10 +12082,10 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B138" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C138" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C138" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D138" s="59" t="s">
         <v>202</v>
@@ -12089,7 +12101,7 @@
         <v>300</v>
       </c>
       <c r="H138" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I138" s="60"/>
       <c r="J138" s="58" t="s">
@@ -12098,10 +12110,10 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C139" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C139" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D139" s="59" t="s">
         <v>205</v>
@@ -12117,17 +12129,17 @@
         <v>180</v>
       </c>
       <c r="H139" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I139" s="60"/>
       <c r="J139" s="58"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C140" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C140" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D140" s="59" t="s">
         <v>205</v>
@@ -12143,17 +12155,17 @@
         <v>200</v>
       </c>
       <c r="H140" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I140" s="60"/>
       <c r="J140" s="58"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C141" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C141" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D141" s="59" t="s">
         <v>207</v>
@@ -12169,17 +12181,17 @@
         <v>180</v>
       </c>
       <c r="H141" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I141" s="60"/>
       <c r="J141" s="58"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B142" s="61" t="s">
+        <v>327</v>
+      </c>
+      <c r="C142" s="58" t="s">
         <v>326</v>
-      </c>
-      <c r="C142" s="58" t="s">
-        <v>325</v>
       </c>
       <c r="D142" s="59" t="s">
         <v>207</v>
@@ -12195,164 +12207,164 @@
         <v>200</v>
       </c>
       <c r="H142" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I142" s="60"/>
       <c r="J142" s="58"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B143" s="57" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C143" s="58" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D143" s="59" t="s">
         <v>210</v>
       </c>
       <c r="E143" s="58"/>
       <c r="F143" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G143" s="55" t="n">
         <f aca="false">IF(Soğuklar!D58="","",Soğuklar!D58)</f>
         <v>40</v>
       </c>
       <c r="H143" s="58" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="I143" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J143" s="58"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="61" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C144" s="58" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D144" s="59" t="s">
         <v>211</v>
       </c>
       <c r="E144" s="58"/>
       <c r="F144" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G144" s="55" t="n">
         <f aca="false">IF(Soğuklar!D59="","",Soğuklar!D59)</f>
         <v>60</v>
       </c>
       <c r="H144" s="58" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="I144" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J144" s="58"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="61" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C145" s="58" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D145" s="59" t="s">
         <v>212</v>
       </c>
       <c r="E145" s="58"/>
       <c r="F145" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G145" s="55" t="n">
         <f aca="false">IF(Soğuklar!D60="","",Soğuklar!D60)</f>
         <v>80</v>
       </c>
       <c r="H145" s="58" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="I145" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J145" s="58"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="61" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C146" s="58" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D146" s="59" t="s">
         <v>213</v>
       </c>
       <c r="E146" s="58"/>
       <c r="F146" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G146" s="55" t="n">
         <f aca="false">IF(Soğuklar!D61="","",Soğuklar!D61)</f>
         <v>120</v>
       </c>
       <c r="H146" s="58" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="I146" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J146" s="58"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B147" s="61" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C147" s="58" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D147" s="59" t="s">
         <v>214</v>
       </c>
       <c r="E147" s="58"/>
       <c r="F147" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G147" s="55" t="n">
         <f aca="false">IF(Soğuklar!D62="","",Soğuklar!D62)</f>
         <v>200</v>
       </c>
       <c r="H147" s="58" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I147" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J147" s="58"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="61" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C148" s="58" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D148" s="59" t="s">
         <v>215</v>
       </c>
       <c r="E148" s="58"/>
       <c r="F148" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G148" s="55" t="n">
         <f aca="false">IF(Soğuklar!D63="","",Soğuklar!D63)</f>
         <v>170</v>
       </c>
       <c r="H148" s="58" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="I148" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J148" s="58"/>
     </row>
@@ -12370,7 +12382,7 @@
         <v>226</v>
       </c>
       <c r="F149" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G149" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E8="","",'Tatlı &amp; Atıştırmalık'!E8)</f>
@@ -12380,7 +12392,7 @@
         <v>340</v>
       </c>
       <c r="I149" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J149" s="58"/>
     </row>
@@ -12398,7 +12410,7 @@
         <v>229</v>
       </c>
       <c r="F150" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G150" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E9="","",'Tatlı &amp; Atıştırmalık'!E9)</f>
@@ -12408,7 +12420,7 @@
         <v>340</v>
       </c>
       <c r="I150" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J150" s="58"/>
     </row>
@@ -12426,7 +12438,7 @@
         <v>232</v>
       </c>
       <c r="F151" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G151" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E10="","",'Tatlı &amp; Atıştırmalık'!E10)</f>
@@ -12436,7 +12448,7 @@
         <v>340</v>
       </c>
       <c r="I151" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J151" s="58"/>
     </row>
@@ -12454,7 +12466,7 @@
         <v>235</v>
       </c>
       <c r="F152" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G152" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E11="","",'Tatlı &amp; Atıştırmalık'!E11)</f>
@@ -12464,7 +12476,7 @@
         <v>340</v>
       </c>
       <c r="I152" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J152" s="58"/>
     </row>
@@ -12482,7 +12494,7 @@
         <v>238</v>
       </c>
       <c r="F153" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G153" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E12="","",'Tatlı &amp; Atıştırmalık'!E12)</f>
@@ -12492,7 +12504,7 @@
         <v>340</v>
       </c>
       <c r="I153" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J153" s="58"/>
     </row>
@@ -12510,7 +12522,7 @@
         <v>241</v>
       </c>
       <c r="F154" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G154" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E13="","",'Tatlı &amp; Atıştırmalık'!E13)</f>
@@ -12520,7 +12532,7 @@
         <v>340</v>
       </c>
       <c r="I154" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J154" s="58"/>
     </row>
@@ -12538,7 +12550,7 @@
         <v>244</v>
       </c>
       <c r="F155" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G155" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E14="","",'Tatlı &amp; Atıştırmalık'!E14)</f>
@@ -12548,7 +12560,7 @@
         <v>340</v>
       </c>
       <c r="I155" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J155" s="58"/>
     </row>
@@ -12566,7 +12578,7 @@
         <v>247</v>
       </c>
       <c r="F156" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G156" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E15="","",'Tatlı &amp; Atıştırmalık'!E15)</f>
@@ -12576,7 +12588,7 @@
         <v>340</v>
       </c>
       <c r="I156" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J156" s="58"/>
     </row>
@@ -12594,7 +12606,7 @@
         <v>251</v>
       </c>
       <c r="F157" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G157" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E18="","",'Tatlı &amp; Atıştırmalık'!E18)</f>
@@ -12604,7 +12616,7 @@
         <v>340</v>
       </c>
       <c r="I157" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J157" s="58"/>
     </row>
@@ -12622,7 +12634,7 @@
         <v>254</v>
       </c>
       <c r="F158" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G158" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E19="","",'Tatlı &amp; Atıştırmalık'!E19)</f>
@@ -12632,7 +12644,7 @@
         <v>340</v>
       </c>
       <c r="I158" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J158" s="58"/>
     </row>
@@ -12650,7 +12662,7 @@
         <v>257</v>
       </c>
       <c r="F159" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G159" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E20="","",'Tatlı &amp; Atıştırmalık'!E20)</f>
@@ -12660,7 +12672,7 @@
         <v>340</v>
       </c>
       <c r="I159" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J159" s="58"/>
     </row>
@@ -12678,7 +12690,7 @@
         <v>260</v>
       </c>
       <c r="F160" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G160" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E21="","",'Tatlı &amp; Atıştırmalık'!E21)</f>
@@ -12688,7 +12700,7 @@
         <v>340</v>
       </c>
       <c r="I160" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J160" s="58"/>
     </row>
@@ -12706,7 +12718,7 @@
         <v>263</v>
       </c>
       <c r="F161" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G161" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E22="","",'Tatlı &amp; Atıştırmalık'!E22)</f>
@@ -12716,7 +12728,7 @@
         <v>340</v>
       </c>
       <c r="I161" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J161" s="58"/>
     </row>
@@ -12734,7 +12746,7 @@
         <v>267</v>
       </c>
       <c r="F162" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G162" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E25="","",'Tatlı &amp; Atıştırmalık'!E25)</f>
@@ -12744,7 +12756,7 @@
         <v>340</v>
       </c>
       <c r="I162" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J162" s="58"/>
     </row>
@@ -12762,7 +12774,7 @@
         <v>269</v>
       </c>
       <c r="F163" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G163" s="55" t="n">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E26="","",'Tatlı &amp; Atıştırmalık'!E26)</f>
@@ -12772,7 +12784,7 @@
         <v>340</v>
       </c>
       <c r="I163" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J163" s="58"/>
     </row>
@@ -12790,7 +12802,7 @@
         <v>272</v>
       </c>
       <c r="F164" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G164" s="55" t="str">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E29="","",'Tatlı &amp; Atıştırmalık'!E29)</f>
@@ -12818,7 +12830,7 @@
         <v>276</v>
       </c>
       <c r="F165" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G165" s="55" t="str">
         <f aca="false">IF('Tatlı &amp; Atıştırmalık'!E30="","",'Tatlı &amp; Atıştırmalık'!E30)</f>
@@ -12846,7 +12858,7 @@
         <v>282</v>
       </c>
       <c r="F166" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G166" s="55" t="n">
         <f aca="false">IF('Kasa Önü'!D8="","",'Kasa Önü'!D8)</f>
@@ -12856,7 +12868,7 @@
         <v>345</v>
       </c>
       <c r="I166" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J166" s="58" t="s">
         <v>283</v>
@@ -12876,7 +12888,7 @@
         <v>285</v>
       </c>
       <c r="F167" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G167" s="55" t="n">
         <f aca="false">IF('Kasa Önü'!D9="","",'Kasa Önü'!D9)</f>
@@ -12886,7 +12898,7 @@
         <v>345</v>
       </c>
       <c r="I167" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J167" s="58" t="s">
         <v>283</v>
@@ -12906,7 +12918,7 @@
         <v>287</v>
       </c>
       <c r="F168" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G168" s="55" t="n">
         <f aca="false">IF('Kasa Önü'!D10="","",'Kasa Önü'!D10)</f>
@@ -12916,7 +12928,7 @@
         <v>345</v>
       </c>
       <c r="I168" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J168" s="58" t="s">
         <v>283</v>
@@ -12936,7 +12948,7 @@
         <v>289</v>
       </c>
       <c r="F169" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G169" s="55" t="n">
         <f aca="false">IF('Kasa Önü'!D11="","",'Kasa Önü'!D11)</f>
@@ -12946,7 +12958,7 @@
         <v>345</v>
       </c>
       <c r="I169" s="60" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="J169" s="58" t="s">
         <v>283</v>
@@ -12964,7 +12976,7 @@
       </c>
       <c r="E170" s="58"/>
       <c r="F170" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G170" s="55" t="n">
         <f aca="false">Sıcaklar!D66</f>
@@ -12990,7 +13002,7 @@
       </c>
       <c r="E171" s="58"/>
       <c r="F171" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G171" s="55" t="n">
         <f aca="false">Sıcaklar!D67</f>
@@ -13016,7 +13028,7 @@
       </c>
       <c r="E172" s="58"/>
       <c r="F172" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G172" s="55" t="n">
         <f aca="false">Sıcaklar!D68</f>
@@ -13042,7 +13054,7 @@
       </c>
       <c r="E173" s="58"/>
       <c r="F173" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G173" s="55" t="n">
         <f aca="false">Sıcaklar!D69</f>
@@ -13068,7 +13080,7 @@
       </c>
       <c r="E174" s="58"/>
       <c r="F174" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G174" s="55" t="n">
         <f aca="false">Sıcaklar!D70</f>
@@ -13094,7 +13106,7 @@
       </c>
       <c r="E175" s="58"/>
       <c r="F175" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G175" s="55" t="n">
         <f aca="false">Soğuklar!D70</f>
@@ -13120,7 +13132,7 @@
       </c>
       <c r="E176" s="58"/>
       <c r="F176" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G176" s="55" t="n">
         <f aca="false">Soğuklar!D71</f>
@@ -13146,7 +13158,7 @@
       </c>
       <c r="E177" s="58"/>
       <c r="F177" s="60" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G177" s="55" t="n">
         <f aca="false">Soğuklar!D72</f>

</xml_diff>